<commit_message>
added new data for Adm. Tribunales
</commit_message>
<xml_diff>
--- a/data/administracion_de_tribunales/tribCasosCrim.xlsx
+++ b/data/administracion_de_tribunales/tribCasosCrim.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlando.hernandez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="2019-2020" sheetId="5" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="2022-2023" sheetId="2" r:id="rId4"/>
     <sheet name="2023-2024" sheetId="3" r:id="rId5"/>
     <sheet name="2024-2025" sheetId="6" r:id="rId6"/>
+    <sheet name="2025-2026" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="14">
   <si>
     <t>Pendiente al inicio</t>
   </si>
@@ -87,9 +88,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -128,11 +129,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" indent="2"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1270,19 +1280,19 @@
         <v>17</v>
       </c>
       <c r="C2" s="1">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D2" s="1">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="E2" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" s="1">
         <v>3</v>
       </c>
       <c r="G2" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2" s="2">
         <v>0</v>
@@ -1291,10 +1301,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K2" s="1">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1302,34 +1312,34 @@
         <v>11</v>
       </c>
       <c r="B3" s="1">
-        <v>1079</v>
+        <v>1060</v>
       </c>
       <c r="C3" s="1">
-        <v>2141</v>
+        <v>2928</v>
       </c>
       <c r="D3" s="1">
-        <v>3220</v>
+        <v>3988</v>
       </c>
       <c r="E3" s="1">
-        <v>1847</v>
+        <v>2638</v>
       </c>
       <c r="F3" s="1">
-        <v>234</v>
+        <v>311</v>
       </c>
       <c r="G3" s="1">
-        <v>408</v>
-      </c>
-      <c r="H3" s="1">
-        <v>4</v>
+        <v>580</v>
+      </c>
+      <c r="H3" s="4">
+        <v>8</v>
       </c>
       <c r="I3" s="1">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="J3" s="1">
-        <v>2508</v>
+        <v>3567</v>
       </c>
       <c r="K3" s="1">
-        <v>984</v>
+        <v>820</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1337,34 +1347,198 @@
         <v>13</v>
       </c>
       <c r="B4" s="1">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C4" s="1">
-        <v>266</v>
+        <v>342</v>
       </c>
       <c r="D4" s="1">
-        <v>391</v>
+        <v>462</v>
       </c>
       <c r="E4" s="1">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F4" s="1">
+        <v>18</v>
+      </c>
+      <c r="G4" s="1">
+        <v>34</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1</v>
+      </c>
+      <c r="J4" s="1">
+        <v>82</v>
+      </c>
+      <c r="K4" s="1">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="58.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.42578125" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>2</v>
+      </c>
+      <c r="K2" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1">
+        <v>820</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1083</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1903</v>
+      </c>
+      <c r="E3" s="1">
+        <v>827</v>
+      </c>
+      <c r="F3" s="1">
+        <v>101</v>
+      </c>
+      <c r="G3" s="2">
+        <v>207</v>
+      </c>
+      <c r="H3" s="5">
+        <v>4</v>
+      </c>
+      <c r="I3" s="2">
+        <v>14</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1153</v>
+      </c>
+      <c r="K3" s="1">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="1">
-        <v>20</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1">
-        <v>2</v>
+      <c r="B4" s="1">
+        <v>66</v>
+      </c>
+      <c r="C4" s="1">
+        <v>99</v>
+      </c>
+      <c r="D4" s="1">
+        <v>165</v>
+      </c>
+      <c r="E4" s="1">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1">
+        <v>7</v>
+      </c>
+      <c r="G4" s="2">
+        <v>6</v>
+      </c>
+      <c r="H4" s="6">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
       </c>
       <c r="J4" s="1">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="K4" s="1">
-        <v>111</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>